<commit_message>
cambios x e y
</commit_message>
<xml_diff>
--- a/participantes.xlsx
+++ b/participantes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Osmar\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0da5e7d2b9b3af27/UNIATLÁNTICO/EIEM8/Certificados-EIEM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{408F2760-2307-43BF-8294-50B542F91E57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{408F2760-2307-43BF-8294-50B542F91E57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E645495-3BB0-464D-A994-01DDE2909A20}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="42">
   <si>
     <t>SILVIO DAVID ACOSTA ACOSTA</t>
   </si>
@@ -140,27 +140,9 @@
     <t>nombre</t>
   </si>
   <si>
-    <t>Rol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Asistente </t>
-  </si>
-  <si>
-    <t>Ponente</t>
-  </si>
-  <si>
     <t>AMOR</t>
   </si>
   <si>
-    <t>PAZ</t>
-  </si>
-  <si>
-    <t>SERVICIO</t>
-  </si>
-  <si>
-    <t>LIDER</t>
-  </si>
-  <si>
     <t>ROMA</t>
   </si>
   <si>
@@ -180,9 +162,6 @@
   </si>
   <si>
     <t>GEOME</t>
-  </si>
-  <si>
-    <t>QUITA</t>
   </si>
   <si>
     <t>Ponecia</t>
@@ -572,15 +551,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="34.81640625" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -588,13 +567,10 @@
         <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>22</v>
       </c>
@@ -602,13 +578,10 @@
         <v>1120654359</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>16</v>
       </c>
@@ -616,10 +589,10 @@
         <v>1107517191</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="7" t="s">
         <v>18</v>
       </c>
@@ -627,13 +600,10 @@
         <v>1142089800</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>19</v>
       </c>
@@ -641,10 +611,10 @@
         <v>1087528105</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="7" t="s">
         <v>25</v>
       </c>
@@ -652,10 +622,10 @@
         <v>1151336537</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
@@ -663,10 +633,10 @@
         <v>1016511325</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>24</v>
       </c>
@@ -674,10 +644,10 @@
         <v>1216852029</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -685,10 +655,10 @@
         <v>1116954607</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>26</v>
       </c>
@@ -696,10 +666,10 @@
         <v>1062911949</v>
       </c>
       <c r="C10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>8</v>
       </c>
@@ -707,10 +677,10 @@
         <v>1200059357</v>
       </c>
       <c r="C11" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="7" t="s">
         <v>15</v>
       </c>
@@ -718,10 +688,10 @@
         <v>1191351967</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -729,10 +699,10 @@
         <v>1191921777</v>
       </c>
       <c r="C13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>7</v>
       </c>
@@ -740,10 +710,10 @@
         <v>1191921777</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="7" t="s">
         <v>17</v>
       </c>
@@ -751,10 +721,10 @@
         <v>1082640575</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
         <v>10</v>
       </c>
@@ -762,10 +732,10 @@
         <v>1066142066</v>
       </c>
       <c r="C16" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>3</v>
       </c>
@@ -773,10 +743,10 @@
         <v>1211224294</v>
       </c>
       <c r="C17" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>6</v>
       </c>
@@ -784,10 +754,10 @@
         <v>1098076877</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
         <v>30</v>
       </c>
@@ -795,10 +765,10 @@
         <v>1029928740</v>
       </c>
       <c r="C19" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>28</v>
       </c>
@@ -806,10 +776,10 @@
         <v>1180591498</v>
       </c>
       <c r="C20" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="7" t="s">
         <v>23</v>
       </c>
@@ -817,10 +787,10 @@
         <v>1103672634</v>
       </c>
       <c r="C21" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="6" t="s">
         <v>21</v>
       </c>
@@ -828,10 +798,10 @@
         <v>1067189873</v>
       </c>
       <c r="C22" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
         <v>14</v>
       </c>
@@ -839,10 +809,10 @@
         <v>1167520326</v>
       </c>
       <c r="C23" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="7" t="s">
         <v>5</v>
       </c>
@@ -850,10 +820,10 @@
         <v>1208001700</v>
       </c>
       <c r="C24" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>29</v>
       </c>
@@ -861,10 +831,10 @@
         <v>1217210939</v>
       </c>
       <c r="C25" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="8" t="s">
         <v>0</v>
       </c>
@@ -872,10 +842,10 @@
         <v>1134633937</v>
       </c>
       <c r="C26" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
         <v>1</v>
       </c>
@@ -883,13 +853,10 @@
         <v>1128929287</v>
       </c>
       <c r="C27" t="s">
-        <v>35</v>
-      </c>
-      <c r="D27" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="6" t="s">
         <v>1</v>
       </c>
@@ -897,13 +864,10 @@
         <v>1128929287</v>
       </c>
       <c r="C28" t="s">
-        <v>35</v>
-      </c>
-      <c r="D28" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="3" t="s">
         <v>1</v>
       </c>
@@ -911,13 +875,10 @@
         <v>1128929287</v>
       </c>
       <c r="C29" t="s">
-        <v>35</v>
-      </c>
-      <c r="D29" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="6" t="s">
         <v>13</v>
       </c>
@@ -925,13 +886,10 @@
         <v>1131939211</v>
       </c>
       <c r="C30" t="s">
-        <v>35</v>
-      </c>
-      <c r="D30" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
         <v>12</v>
       </c>
@@ -939,10 +897,10 @@
         <v>1036321978</v>
       </c>
       <c r="C31" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="3" t="s">
         <v>27</v>
       </c>
@@ -950,13 +908,10 @@
         <v>1120654359</v>
       </c>
       <c r="C32" t="s">
-        <v>35</v>
-      </c>
-      <c r="D32" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
         <v>4</v>
       </c>
@@ -964,13 +919,10 @@
         <v>1120654359</v>
       </c>
       <c r="C33" t="s">
-        <v>35</v>
-      </c>
-      <c r="D33" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>4</v>
       </c>
@@ -978,13 +930,10 @@
         <v>1120654359</v>
       </c>
       <c r="C34" t="s">
-        <v>35</v>
-      </c>
-      <c r="D34" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="3" t="s">
         <v>4</v>
       </c>
@@ -992,13 +941,10 @@
         <v>1120654359</v>
       </c>
       <c r="C35" t="s">
-        <v>35</v>
-      </c>
-      <c r="D35" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="6" t="s">
         <v>4</v>
       </c>
@@ -1008,11 +954,8 @@
       <c r="C36" t="s">
         <v>35</v>
       </c>
-      <c r="D36" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
         <v>4</v>
       </c>
@@ -1020,13 +963,10 @@
         <v>1120654359</v>
       </c>
       <c r="C37" t="s">
-        <v>35</v>
-      </c>
-      <c r="D37" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="7" t="s">
         <v>9</v>
       </c>

</xml_diff>